<commit_message>
use unmerged original card sheet for ledger rows
</commit_message>
<xml_diff>
--- a/backend/app/modules/safety_ledgers/templates/company-card-template.xlsx
+++ b/backend/app/modules/safety_ledgers/templates/company-card-template.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JSI\besma-safety-ledgers-deploy\backend\app\modules\safety_ledgers\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609EFDDE-D517-47FA-851C-64E3BE6F33C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD18F84-DB12-4FB8-9605-176DBE2BFC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3EB6DA63-AEF3-4714-B578-A35BA89CE9B3}"/>
   </bookViews>
   <sheets>
-    <sheet name="template" sheetId="2" r:id="rId1"/>
+    <sheet name="template" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_" hidden="1">#REF!</definedName>
@@ -4160,7 +4160,6 @@
     <definedName name="DD" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="ddd">#REF!</definedName>
     <definedName name="dddd" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
-    <definedName name="DDDDA" localSheetId="0">BlankMacro1</definedName>
     <definedName name="DDDDA">BlankMacro1</definedName>
     <definedName name="ddddd" hidden="1">#REF!</definedName>
     <definedName name="dddddd" hidden="1">{#N/A,#N/A,FALSE,"하중 계산 (1)";#N/A,#N/A,FALSE,"토압계수계산";#N/A,#N/A,FALSE,"횡토압계산";#N/A,#N/A,FALSE,"전도에 대한 안정";#N/A,#N/A,FALSE,"활동에 대한 안정";#N/A,#N/A,FALSE,"지지력 검토";#N/A,#N/A,FALSE,"PILE 계산";#N/A,#N/A,FALSE,"PILE계산결과";#N/A,#N/A,FALSE,"PILE검토";#N/A,#N/A,FALSE,"벽체의 설계"}</definedName>
@@ -4174,9 +4173,7 @@
     <definedName name="DDFD" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="DDFRE" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="DDR">#REF!</definedName>
-    <definedName name="DDS" localSheetId="0">BlankMacro1</definedName>
     <definedName name="DDS">BlankMacro1</definedName>
-    <definedName name="DDW" localSheetId="0">BlankMacro1</definedName>
     <definedName name="DDW">BlankMacro1</definedName>
     <definedName name="DE" hidden="1">#REF!</definedName>
     <definedName name="DEC.GH">#REF!</definedName>
@@ -4239,7 +4236,6 @@
     <definedName name="DirectLabor" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="DirectLobor" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="dj" hidden="1">{#N/A,#N/A,FALSE,"하중 계산 (1)";#N/A,#N/A,FALSE,"토압계수계산";#N/A,#N/A,FALSE,"횡토압계산";#N/A,#N/A,FALSE,"전도에 대한 안정";#N/A,#N/A,FALSE,"활동에 대한 안정";#N/A,#N/A,FALSE,"지지력 검토";#N/A,#N/A,FALSE,"PILE 계산";#N/A,#N/A,FALSE,"PILE계산결과";#N/A,#N/A,FALSE,"PILE검토";#N/A,#N/A,FALSE,"벽체의 설계"}</definedName>
-    <definedName name="DJDJ" localSheetId="0">BlankMacro1</definedName>
     <definedName name="DJDJ">BlankMacro1</definedName>
     <definedName name="djdlof" hidden="1">{#N/A,#N/A,FALSE,"지침";#N/A,#N/A,FALSE,"환경분석";#N/A,#N/A,FALSE,"Sheet16"}</definedName>
     <definedName name="djfgkhfgh" hidden="1">{#N/A,#N/A,FALSE,"운반시간"}</definedName>
@@ -4251,15 +4247,12 @@
     <definedName name="DJYDTYJ" hidden="1">#REF!</definedName>
     <definedName name="dk" hidden="1">{#N/A,#N/A,FALSE,"하중 계산 (1)";#N/A,#N/A,FALSE,"토압계수계산";#N/A,#N/A,FALSE,"횡토압계산";#N/A,#N/A,FALSE,"전도에 대한 안정";#N/A,#N/A,FALSE,"활동에 대한 안정";#N/A,#N/A,FALSE,"지지력 검토";#N/A,#N/A,FALSE,"PILE 계산";#N/A,#N/A,FALSE,"PILE계산결과";#N/A,#N/A,FALSE,"PILE검토";#N/A,#N/A,FALSE,"벽체의 설계"}</definedName>
     <definedName name="DKC" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
-    <definedName name="DKD" localSheetId="0">BlankMacro1</definedName>
     <definedName name="DKD">BlankMacro1</definedName>
     <definedName name="dkdjhlajf" hidden="1">{#N/A,#N/A,FALSE,"BE-001";#N/A,#N/A,FALSE,"CA-001";#N/A,#N/A,FALSE,"CY-001";#N/A,#N/A,FALSE,"CU-001";#N/A,#N/A,FALSE,"D-001";#N/A,#N/A,FALSE,"D-002";#N/A,#N/A,FALSE,"DH-001";#N/A,#N/A,FALSE,"DU-001";#N/A,#N/A,FALSE,"E-001";#N/A,#N/A,FALSE,"E-002";#N/A,#N/A,FALSE,"E-003";#N/A,#N/A,FALSE,"E-004";#N/A,#N/A,FALSE,"E-005";#N/A,#N/A,FALSE,"E-006";#N/A,#N/A,FALSE,"E-007";#N/A,#N/A,FALSE,"EH-001";#N/A,#N/A,FALSE,"EL-001";#N/A,#N/A,FALSE,"F-001";#N/A,#N/A,FALSE,"F-002";#N/A,#N/A,FALSE,"FI-001";#N/A,#N/A,FALSE,"J-001";#N/A,#N/A,FALSE,"J-002";#N/A,#N/A,FALSE,"N2-001";#N/A,#N/A,FALSE,"PT-001";#N/A,#N/A,FALSE,"R-001";#N/A,#N/A,FALSE,"SI-001";#N/A,#N/A,FALSE,"SM-001";#N/A,#N/A,FALSE,"T-001";#N/A,#N/A,FALSE,"T-002";#N/A,#N/A,FALSE,"T-003";#N/A,#N/A,FALSE,"TO-001";#N/A,#N/A,FALSE,"X-002";#N/A,#N/A,FALSE,"X-003";#N/A,#N/A,FALSE,"S_STR"}</definedName>
     <definedName name="dkdkdkdkd" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="dkdkoo">#REF!</definedName>
-    <definedName name="DKE" localSheetId="0">BlankMacro1</definedName>
     <definedName name="DKE">BlankMacro1</definedName>
     <definedName name="DKFK">[0]!DKFK</definedName>
-    <definedName name="DKJFL" localSheetId="0">BlankMacro1</definedName>
     <definedName name="DKJFL">BlankMacro1</definedName>
     <definedName name="dkjhgfhfd">#REF!</definedName>
     <definedName name="DKSG" hidden="1">#REF!</definedName>
@@ -4336,7 +4329,6 @@
     <definedName name="DW">{"'용역비'!$A$4:$C$8"}</definedName>
     <definedName name="DWD" hidden="1">{#N/A,#N/A,FALSE,"하중 계산 (1)";#N/A,#N/A,FALSE,"토압계수계산";#N/A,#N/A,FALSE,"횡토압계산";#N/A,#N/A,FALSE,"전도에 대한 안정";#N/A,#N/A,FALSE,"활동에 대한 안정";#N/A,#N/A,FALSE,"지지력 검토";#N/A,#N/A,FALSE,"PILE 계산";#N/A,#N/A,FALSE,"PILE계산결과";#N/A,#N/A,FALSE,"PILE검토";#N/A,#N/A,FALSE,"벽체의 설계"}</definedName>
     <definedName name="dweydfgh" hidden="1">{#N/A,#N/A,FALSE,"배수1"}</definedName>
-    <definedName name="DWS" localSheetId="0">BlankMacro1</definedName>
     <definedName name="DWS">BlankMacro1</definedName>
     <definedName name="dx_shape">#REF!</definedName>
     <definedName name="DXFFFS" hidden="1">{#N/A,#N/A,FALSE,"지침";#N/A,#N/A,FALSE,"환경분석";#N/A,#N/A,FALSE,"Sheet16"}</definedName>
@@ -4631,7 +4623,6 @@
     <definedName name="FGGHH" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="fgh" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="fghfgh" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
-    <definedName name="fghgh" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="fghgh">[0]!영광원자력5,#REF!</definedName>
     <definedName name="fghjfjg" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="fghkfgj" hidden="1">{#N/A,#N/A,FALSE,"조골재"}</definedName>
@@ -4798,7 +4789,6 @@
     <definedName name="gbi_s_so_1">#REF!</definedName>
     <definedName name="gbi_s_so_2">#REF!</definedName>
     <definedName name="GBI_S_YEO">#REF!</definedName>
-    <definedName name="gcfj" localSheetId="0">BlankMacro1</definedName>
     <definedName name="gcfj">BlankMacro1</definedName>
     <definedName name="GCODE">#N/A</definedName>
     <definedName name="GDBBNDF" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
@@ -5223,7 +5213,6 @@
     <definedName name="LLDIEKKS" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="LLKD" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="LLL" hidden="1">#REF!</definedName>
-    <definedName name="LLLL" localSheetId="0">BlankMacro1</definedName>
     <definedName name="LLLL">BlankMacro1</definedName>
     <definedName name="LLLLL" hidden="1">#REF!</definedName>
     <definedName name="LLLS" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
@@ -5231,7 +5220,6 @@
     <definedName name="LLM">#REF!</definedName>
     <definedName name="LLSIEKDKD" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="LLSKEIE" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="LOB공정표" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="LOB공정표">[0]!영광원자력5,#REF!</definedName>
     <definedName name="lod" hidden="1">#N/A</definedName>
     <definedName name="loe">{"'5'!$A$1:$BB$147"}</definedName>
@@ -5584,7 +5572,6 @@
     <definedName name="PSKS13C6LRTOR3C76R62C87RTM1TB0T">#REF!</definedName>
     <definedName name="PSUL">#REF!</definedName>
     <definedName name="pu" hidden="1">{#N/A,#N/A,FALSE,"표지"}</definedName>
-    <definedName name="pump" localSheetId="0">BlankMacro1</definedName>
     <definedName name="pump">BlankMacro1</definedName>
     <definedName name="Pump1">#REF!</definedName>
     <definedName name="Pump2">#REF!</definedName>
@@ -5600,7 +5587,6 @@
     <definedName name="qedgagsd" hidden="1">#REF!</definedName>
     <definedName name="QEFQEF" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="qewewre" hidden="1">#REF!</definedName>
-    <definedName name="qewqwe" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="qewqwe">[0]!영광원자력5,#REF!</definedName>
     <definedName name="Qe앨">#REF!</definedName>
     <definedName name="QFFGGB" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
@@ -5627,7 +5613,6 @@
     <definedName name="qsaaaa" hidden="1">#REF!</definedName>
     <definedName name="QSR">#REF!</definedName>
     <definedName name="QSS">#REF!</definedName>
-    <definedName name="qtw" localSheetId="0">BlankMacro1</definedName>
     <definedName name="qtw">BlankMacro1</definedName>
     <definedName name="QTY">#N/A</definedName>
     <definedName name="qu">#REF!</definedName>
@@ -5661,7 +5646,6 @@
     <definedName name="RawAgencyPrice">#REF!</definedName>
     <definedName name="RBData">#REF!</definedName>
     <definedName name="re_bar">#REF!</definedName>
-    <definedName name="RE2WERT" localSheetId="0">BlankMacro1</definedName>
     <definedName name="RE2WERT">BlankMacro1</definedName>
     <definedName name="_xlnm.Recorder">#REF!</definedName>
     <definedName name="REG" hidden="1">#REF!</definedName>
@@ -5689,9 +5673,7 @@
     <definedName name="RHDK" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="RHKDWN" hidden="1">{#N/A,#N/A,FALSE,"운반시간"}</definedName>
     <definedName name="RISK">{"'con_010'!$A$1:$AN$63"}</definedName>
-    <definedName name="RJRJ" localSheetId="0">BlankMacro1</definedName>
     <definedName name="RJRJ">BlankMacro1</definedName>
-    <definedName name="RJRKJRKJR" localSheetId="0">BlankMacro1</definedName>
     <definedName name="RJRKJRKJR">BlankMacro1</definedName>
     <definedName name="rk" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="rka">{"'집계표'!$A$1:$F$40"}</definedName>
@@ -5702,7 +5684,6 @@
     <definedName name="RKSK" hidden="1">{#N/A,#N/A,FALSE,"집계";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"터빈집계";#N/A,#N/A,FALSE,"터빈내역";#N/A,#N/A,FALSE,"주제어집계";#N/A,#N/A,FALSE,"주제어내역";#N/A,#N/A,FALSE,"보일러집계";#N/A,#N/A,FALSE,"보일러내역";#N/A,#N/A,FALSE,"별표19";#N/A,#N/A,FALSE,"정산신규품";#N/A,#N/A,FALSE,"신규별표";#N/A,#N/A,FALSE,"골재 ";#N/A,#N/A,FALSE,"운반비"}</definedName>
     <definedName name="RKSKEK" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="rkstjs">[0]!rkstjs</definedName>
-    <definedName name="RL" localSheetId="0">BlankMacro1</definedName>
     <definedName name="RL">BlankMacro1</definedName>
     <definedName name="RLA" hidden="1">{#N/A,#N/A,FALSE,"양식(을)"}</definedName>
     <definedName name="RLAGHKSCJF" hidden="1">#REF!</definedName>
@@ -5713,7 +5694,6 @@
     <definedName name="RMRM">#REF!</definedName>
     <definedName name="RNAO">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="RNSEO" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
-    <definedName name="ro" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ro">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ROC">{"'QuotationCRPaint (3)'!$A$12:$B$15"}</definedName>
     <definedName name="ROOF_AND_DRAIN_WORKS">#REF!</definedName>
@@ -5876,7 +5856,6 @@
     <definedName name="SHEET100" hidden="1">#REF!</definedName>
     <definedName name="SHEET3">{"'NOTES2'!$G$9:$J$27"}</definedName>
     <definedName name="SHEET56">#REF!</definedName>
-    <definedName name="SHEET8" localSheetId="0">BlankMacro1</definedName>
     <definedName name="SHEET8">BlankMacro1</definedName>
     <definedName name="SHH" hidden="1">{#N/A,#N/A,FALSE,"주간공정";#N/A,#N/A,FALSE,"주간보고";#N/A,#N/A,FALSE,"주간공정표"}</definedName>
     <definedName name="SHOP">{"'표지'!$B$5"}</definedName>
@@ -5910,7 +5889,6 @@
     <definedName name="SNVANFENWFE" hidden="1">{#N/A,#N/A,FALSE,"ENG'G(보호계전기)"}</definedName>
     <definedName name="soc">[0]!soc</definedName>
     <definedName name="SOCKET">#REF!</definedName>
-    <definedName name="SODURTJ" localSheetId="0">Dlog_Show</definedName>
     <definedName name="SODURTJ">Dlog_Show</definedName>
     <definedName name="solver_cvg" hidden="1">0.001</definedName>
     <definedName name="solver_drv" hidden="1">1</definedName>
@@ -5952,7 +5930,6 @@
     <definedName name="SSSS">#REF!</definedName>
     <definedName name="sssscda" hidden="1">#REF!</definedName>
     <definedName name="SSSSS" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="sssssssssss" localSheetId="0">BlankMacro1</definedName>
     <definedName name="sssssssssss">BlankMacro1</definedName>
     <definedName name="sssw">#REF!</definedName>
     <definedName name="SSVSS" hidden="1">#REF!</definedName>
@@ -5965,7 +5942,6 @@
     <definedName name="Story_Total">#REF!</definedName>
     <definedName name="Struct_Type">#REF!</definedName>
     <definedName name="STS">{"'용역비'!$A$4:$C$8"}</definedName>
-    <definedName name="ST산출" localSheetId="0">[0]!BlankMacro1</definedName>
     <definedName name="ST산출">[0]!BlankMacro1</definedName>
     <definedName name="SUB" hidden="1">#REF!</definedName>
     <definedName name="SubDic">#REF!</definedName>
@@ -6134,7 +6110,6 @@
     <definedName name="Ted">#REF!</definedName>
     <definedName name="Tel">#REF!</definedName>
     <definedName name="TEMP" hidden="1">#REF!</definedName>
-    <definedName name="temp2" localSheetId="0">BlankMacro1</definedName>
     <definedName name="temp2">BlankMacro1</definedName>
     <definedName name="temporary" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="TEMPORARY_WORKS">#REF!</definedName>
@@ -6546,7 +6521,6 @@
     <definedName name="WT">#REF!</definedName>
     <definedName name="wtr">#REF!</definedName>
     <definedName name="wuy">{"'용역비'!$A$4:$C$8"}</definedName>
-    <definedName name="WV" localSheetId="0">BlankMacro1</definedName>
     <definedName name="WV">BlankMacro1</definedName>
     <definedName name="WW">#REF!</definedName>
     <definedName name="WWD">#REF!</definedName>
@@ -6667,7 +6641,6 @@
     <definedName name="ㄱㄷㄱㄷ" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="ㄱㄷ쇼" hidden="1">#REF!</definedName>
     <definedName name="ㄱㄷㅈ" hidden="1">#REF!</definedName>
-    <definedName name="ㄱㄷㅈㄱ" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ㄱㄷㅈㄱ">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ㄱㄷㅈㅄㄷ" hidden="1">#REF!</definedName>
     <definedName name="ㄱㄷ죠" hidden="1">#REF!</definedName>
@@ -6743,7 +6716,6 @@
     <definedName name="간" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="간노">#REF!</definedName>
     <definedName name="간노_1">#REF!</definedName>
-    <definedName name="간선변경" localSheetId="0">BlankMacro1</definedName>
     <definedName name="간선변경">BlankMacro1</definedName>
     <definedName name="간저비3" hidden="1">{#N/A,#N/A,FALSE,"갑지";#N/A,#N/A,FALSE,"개요";#N/A,#N/A,FALSE,"비목별";#N/A,#N/A,FALSE,"건물별";#N/A,#N/A,FALSE,"기구표";#N/A,#N/A,FALSE,"직원투입"}</definedName>
     <definedName name="간접">#REF!</definedName>
@@ -6753,7 +6725,6 @@
     <definedName name="간접비1" hidden="1">{#N/A,#N/A,FALSE,"갑지";#N/A,#N/A,FALSE,"개요";#N/A,#N/A,FALSE,"비목별";#N/A,#N/A,FALSE,"건물별";#N/A,#N/A,FALSE,"기구표";#N/A,#N/A,FALSE,"직원투입"}</definedName>
     <definedName name="간접비내역">#REF!</definedName>
     <definedName name="간접재료비">#REF!</definedName>
-    <definedName name="간지" localSheetId="0">BlankMacro1</definedName>
     <definedName name="간지">BlankMacro1</definedName>
     <definedName name="감" hidden="1">#REF!</definedName>
     <definedName name="감R10">#REF!</definedName>
@@ -6766,14 +6737,12 @@
     <definedName name="감독조서" hidden="1">{#N/A,#N/A,FALSE,"집계표"}</definedName>
     <definedName name="감리상주" hidden="1">{#N/A,#N/A,FALSE,"지침";#N/A,#N/A,FALSE,"환경분석";#N/A,#N/A,FALSE,"Sheet16"}</definedName>
     <definedName name="감마new" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
-    <definedName name="감자" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="감자">[0]!영광원자력5,#REF!</definedName>
     <definedName name="갑">#REF!</definedName>
     <definedName name="갑지" hidden="1">#REF!</definedName>
     <definedName name="갑지1" hidden="1">#REF!</definedName>
     <definedName name="갑지2" hidden="1">#REF!</definedName>
     <definedName name="갑지3" hidden="1">#REF!</definedName>
-    <definedName name="갑지도급비교" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="갑지도급비교">[0]!영광원자력5,#REF!</definedName>
     <definedName name="강104">#REF!</definedName>
     <definedName name="강6">#REF!</definedName>
@@ -6867,7 +6836,6 @@
     <definedName name="견적2" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="견적3" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="견적4" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="견적LIST" localSheetId="0">Dlog_Show</definedName>
     <definedName name="견적LIST">Dlog_Show</definedName>
     <definedName name="견적SHEET" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="견적갑">#REF!</definedName>
@@ -6883,12 +6851,10 @@
     <definedName name="견적실단가적용" hidden="1">{#N/A,#N/A,TRUE,"토적및재료집계";#N/A,#N/A,TRUE,"토적및재료집계";#N/A,#N/A,TRUE,"단위량"}</definedName>
     <definedName name="견적예가" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="견적의뢰">#REF!</definedName>
-    <definedName name="견적조" localSheetId="0">BlankMacro1</definedName>
     <definedName name="견적조">BlankMacro1</definedName>
     <definedName name="견적조건" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="견적조건1">#REF!</definedName>
     <definedName name="견적조건2" hidden="1">#REF!</definedName>
-    <definedName name="견적조건22" localSheetId="0">BlankMacro1</definedName>
     <definedName name="견적조건22">BlankMacro1</definedName>
     <definedName name="견적조건3">{"Book1","도곡1실행.xls"}</definedName>
     <definedName name="견적조건8" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
@@ -6935,7 +6901,6 @@
     <definedName name="경상자재">{"'집계표'!$A$1:$F$40"}</definedName>
     <definedName name="경수" hidden="1">{#N/A,#N/A,FALSE,"도급대비시행율";#N/A,#N/A,FALSE,"결의서";#N/A,#N/A,FALSE,"내역서";#N/A,#N/A,FALSE,"도급예상"}</definedName>
     <definedName name="경수을지" hidden="1">{#N/A,#N/A,FALSE,"물가변동";#N/A,#N/A,FALSE,"집계";#N/A,#N/A,FALSE,"도급집계";#N/A,#N/A,FALSE,"예산서";#N/A,#N/A,FALSE,"터빈";#N/A,#N/A,FALSE,"보일러";#N/A,#N/A,FALSE,"품셈";#N/A,#N/A,FALSE,"부표";#N/A,#N/A,FALSE,"적용노임";#N/A,#N/A,FALSE,"장비노임";#N/A,#N/A,FALSE,"정산품질";#N/A,#N/A,FALSE,"신규별표";#N/A,#N/A,FALSE,"정산신규품";#N/A,#N/A,FALSE,"ESC별표"}</definedName>
-    <definedName name="경순" localSheetId="0">BlankMacro1</definedName>
     <definedName name="경순">BlankMacro1</definedName>
     <definedName name="경용">#REF!</definedName>
     <definedName name="경우" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
@@ -6974,7 +6939,6 @@
     <definedName name="고령" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="고문" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="고압">#REF!</definedName>
-    <definedName name="고양시성라공원" localSheetId="0">Dlog_Show</definedName>
     <definedName name="고양시성라공원">Dlog_Show</definedName>
     <definedName name="고용">#REF!</definedName>
     <definedName name="고용보험" hidden="1">#REF!</definedName>
@@ -7163,9 +7127,7 @@
     <definedName name="구래">{"'표지'!$B$5"}</definedName>
     <definedName name="구리" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="구부" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
-    <definedName name="구분" localSheetId="0">BlankMacro1</definedName>
     <definedName name="구분">BlankMacro1</definedName>
-    <definedName name="구분1" localSheetId="0">BlankMacro1</definedName>
     <definedName name="구분1">BlankMacro1</definedName>
     <definedName name="구사업계획">#REF!</definedName>
     <definedName name="구산갑지" hidden="1">#REF!</definedName>
@@ -7216,7 +7178,6 @@
     <definedName name="금액합계">#REF!</definedName>
     <definedName name="금오관" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="금융비용" hidden="1">{#N/A,#N/A,FALSE,"조골재"}</definedName>
-    <definedName name="급여표" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="급여표">[0]!영광원자력5,#REF!</definedName>
     <definedName name="기" hidden="1">{#N/A,#N/A,TRUE,"표지";#N/A,#N/A,TRUE,"목차";#N/A,#N/A,TRUE,"1.0일반사항";#N/A,#N/A,TRUE,"2.0공급범위";#N/A,#N/A,TRUE,"3.0현장조건";#N/A,#N/A,TRUE,"4.0적용규격및표준";#N/A,#N/A,TRUE,"5.0요구조건";#N/A,#N/A,TRUE,"6.0시험및검사";#N/A,#N/A,TRUE,"7.0성능보장";#N/A,#N/A,TRUE,"8.0도장";#N/A,#N/A,TRUE,"9.0운송및납품";#N/A,#N/A,TRUE,"10예비품및공구";#N/A,#N/A,TRUE,"11대안";#N/A,#N/A,TRUE,"12제출자료";#N/A,#N/A,TRUE,"13입찰서양식";#N/A,#N/A,TRUE,"14첨부"}</definedName>
     <definedName name="기124">#REF!</definedName>
@@ -7258,7 +7219,6 @@
     <definedName name="기성산출서" hidden="1">{#N/A,#N/A,TRUE,"960318-1";#N/A,#N/A,TRUE,"960318-2";#N/A,#N/A,TRUE,"960318-3"}</definedName>
     <definedName name="기성업체" hidden="1">{#N/A,#N/A,FALSE,"양식(을)"}</definedName>
     <definedName name="기성집계">{"Book1","예술의전당.xls"}</definedName>
-    <definedName name="기성품" localSheetId="0">BlankMacro1</definedName>
     <definedName name="기성품">BlankMacro1</definedName>
     <definedName name="기성화일" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="기술" hidden="1">{#N/A,#N/A,FALSE,"부대1"}</definedName>
@@ -7369,7 +7329,6 @@
     <definedName name="ㄴㄴㄴㄴㄴㄴㄴㄴㄴㄴㄴㄴㄴㄴㄴㄴㄴ" hidden="1">#REF!</definedName>
     <definedName name="ㄴㄴㄴㄴㅇ">#N/A</definedName>
     <definedName name="ㄴㄴㄴㅇㅁ" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
-    <definedName name="ㄴㄴㅁㅁㅁㅁㅁㄴ" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ㄴㄴㅁㅁㅁㅁㅁㄴ">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ㄴㄴㅇ">#REF!</definedName>
     <definedName name="ㄴㄷㄹ" hidden="1">{#N/A,#N/A,FALSE,"Sheet1"}</definedName>
@@ -7488,7 +7447,6 @@
     <definedName name="ㄴ옭ㅎㅇㄹ" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="ㄴ젖" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="ㄴㅊㅎㄷㅈ" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
-    <definedName name="ㄴㅍ" localSheetId="0">[0]!BlankMacro1</definedName>
     <definedName name="ㄴㅍ">[0]!BlankMacro1</definedName>
     <definedName name="ㄴ호" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="ㄴ홎고" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
@@ -7518,7 +7476,6 @@
     <definedName name="난방">{"서울냉천 3차( 5. 6-7).xls","Sheet1"}</definedName>
     <definedName name="남근학이천년">#REF!</definedName>
     <definedName name="남남" hidden="1">#REF!</definedName>
-    <definedName name="남덕" localSheetId="0">BlankMacro1</definedName>
     <definedName name="남덕">BlankMacro1</definedName>
     <definedName name="남서울문화체육관" hidden="1">{#N/A,#N/A,FALSE,"앞";#N/A,#N/A,FALSE,"앞";#N/A,#N/A,FALSE,"목차";#N/A,#N/A,FALSE,"1";#N/A,#N/A,FALSE,"갑지";#N/A,#N/A,FALSE,"2";#N/A,#N/A,FALSE,"개요";#N/A,#N/A,FALSE,"개요2";#N/A,#N/A,FALSE,"3";#N/A,#N/A,FALSE,"총괄";#N/A,#N/A,FALSE,"선금";#N/A,#N/A,FALSE,"4";#N/A,#N/A,FALSE,"방법";#N/A,#N/A,FALSE,"5";#N/A,#N/A,FALSE,"k";#N/A,#N/A,FALSE,"6";#N/A,#N/A,FALSE,"지수";#N/A,#N/A,FALSE,"7";#N/A,#N/A,FALSE,"노";#N/A,#N/A,FALSE,"경";#N/A,#N/A,FALSE,"재";#N/A,#N/A,FALSE,"산";#N/A,#N/A,FALSE,"안";#N/A,#N/A,FALSE,"8";#N/A,#N/A,FALSE,"계수";#N/A,#N/A,FALSE,"9";#N/A,#N/A,FALSE,"비목";#N/A,#N/A,FALSE,"10";#N/A,#N/A,FALSE,"집계"}</definedName>
     <definedName name="남양">#REF!</definedName>
@@ -7609,9 +7566,7 @@
     <definedName name="노원문화" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="노원문화1" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="노임">#REF!</definedName>
-    <definedName name="노임1" localSheetId="0">BlankMacro1</definedName>
     <definedName name="노임1">BlankMacro1</definedName>
-    <definedName name="노임2" localSheetId="0">BlankMacro1</definedName>
     <definedName name="노임2">BlankMacro1</definedName>
     <definedName name="노임단가">#REF!</definedName>
     <definedName name="노임단가1">#REF!</definedName>
@@ -7815,7 +7770,6 @@
     <definedName name="대비" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="대비2">{"Book1","도곡1실행.xls"}</definedName>
     <definedName name="대비5">#N/A</definedName>
-    <definedName name="대비표" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="대비표">[0]!영광원자력5,#REF!</definedName>
     <definedName name="대상" hidden="1">{#N/A,#N/A,FALSE,"2~8번"}</definedName>
     <definedName name="대상아파트24">#REF!</definedName>
@@ -7967,7 +7921,6 @@
     <definedName name="등R4">#REF!</definedName>
     <definedName name="등R6">#REF!</definedName>
     <definedName name="등R8">#REF!</definedName>
-    <definedName name="등기구" localSheetId="0">BlankMacro1</definedName>
     <definedName name="등기구">BlankMacro1</definedName>
     <definedName name="등용구분">[0]!등용구분</definedName>
     <definedName name="등주높이">[0]!등주높이</definedName>
@@ -7979,7 +7932,6 @@
     <definedName name="때죽R8">#REF!</definedName>
     <definedName name="떠">#N/A</definedName>
     <definedName name="떠ㅗㄱ" hidden="1">{#N/A,#N/A,FALSE,"표지"}</definedName>
-    <definedName name="또" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="또">[0]!영광원자력5,#REF!</definedName>
     <definedName name="똑" hidden="1">{#N/A,#N/A,TRUE,"1";#N/A,#N/A,TRUE,"2";#N/A,#N/A,TRUE,"3";#N/A,#N/A,TRUE,"4";#N/A,#N/A,TRUE,"5";#N/A,#N/A,TRUE,"6";#N/A,#N/A,TRUE,"7"}</definedName>
     <definedName name="똥">{"'5'!$A$1:$BB$147"}</definedName>
@@ -8025,7 +7977,6 @@
     <definedName name="ㄹㅇㄹㅇㄹㅇㄹㅇ">#N/A</definedName>
     <definedName name="ㄹㅇㄹㅈㄷㅊ" hidden="1">#REF!</definedName>
     <definedName name="ㄹㅇㄹ호" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
-    <definedName name="ㄹㅇㅁㄴ" localSheetId="0">BlankMacro1</definedName>
     <definedName name="ㄹㅇㅁㄴ">BlankMacro1</definedName>
     <definedName name="ㄹㅇㅁㄴㄹ" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="ㄹㅇㅇㄹ노" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
@@ -8097,7 +8048,6 @@
     <definedName name="래" hidden="1">{#N/A,#N/A,FALSE,"변경관리예산";#N/A,#N/A,FALSE,"변경장비예산";#N/A,#N/A,FALSE,"변경준설예산";#N/A,#N/A,FALSE,"변경철구예산"}</definedName>
     <definedName name="래그" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="랴" hidden="1">{#N/A,#N/A,FALSE,"예상손익";#N/A,#N/A,FALSE,"관리분석";#N/A,#N/A,FALSE,"장비분석";#N/A,#N/A,FALSE,"준설분석";#N/A,#N/A,FALSE,"철구분석"}</definedName>
-    <definedName name="러러러" localSheetId="0">BlankMacro1</definedName>
     <definedName name="러러러">BlankMacro1</definedName>
     <definedName name="러헐" hidden="1">{#N/A,#N/A,FALSE,"도급대비시행율";#N/A,#N/A,FALSE,"결의서";#N/A,#N/A,FALSE,"내역서";#N/A,#N/A,FALSE,"도급예상"}</definedName>
     <definedName name="러ㅛㄷㄷㅅ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
@@ -8133,7 +8083,6 @@
     <definedName name="료ㅏㅓ사ㅕㅕ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="료ㅕㅗ뮤ㅗ5곰ㅅ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="루훓ㅎ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="룰루랄라" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="룰루랄라">[0]!영광원자력5,#REF!</definedName>
     <definedName name="룸" hidden="1">{#N/A,#N/A,FALSE,"사업총괄";#N/A,#N/A,FALSE,"장비사업";#N/A,#N/A,FALSE,"철구사업";#N/A,#N/A,FALSE,"준설사업"}</definedName>
     <definedName name="류">{"서울냉천 3차( 5. 6-7).xls","Sheet1"}</definedName>
@@ -8330,7 +8279,6 @@
     <definedName name="막">#REF!</definedName>
     <definedName name="만득이" hidden="1">{#N/A,#N/A,FALSE,"2~8번"}</definedName>
     <definedName name="만수" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
-    <definedName name="말" localSheetId="0">BlankMacro1</definedName>
     <definedName name="말">BlankMacro1</definedName>
     <definedName name="말발도리1003">#REF!</definedName>
     <definedName name="말발도리1204">#REF!</definedName>
@@ -8424,9 +8372,7 @@
     <definedName name="목차" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
     <definedName name="목차9" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="목차로">#REF!</definedName>
-    <definedName name="목포" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="목포">[0]!영광원자력5,#REF!</definedName>
-    <definedName name="목포공항" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="목포공항">[0]!영광원자력5,#REF!</definedName>
     <definedName name="목표관리">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="목표실행">[0]!목표실행</definedName>
@@ -8448,7 +8394,6 @@
     <definedName name="무궁화2006">#REF!</definedName>
     <definedName name="무늬강판_제작_설치">#REF!</definedName>
     <definedName name="무늬강판제작설치">#REF!</definedName>
-    <definedName name="무대조명일위대가" localSheetId="0">BlankMacro1</definedName>
     <definedName name="무대조명일위대가">BlankMacro1</definedName>
     <definedName name="무인대비">#REF!</definedName>
     <definedName name="문">{"'5'!$A$1:$BB$147"}</definedName>
@@ -8543,7 +8488,6 @@
     <definedName name="ㅂㅍ" hidden="1">{#N/A,#N/A,FALSE,"하중 계산 (1)";#N/A,#N/A,FALSE,"토압계수계산";#N/A,#N/A,FALSE,"횡토압계산";#N/A,#N/A,FALSE,"전도에 대한 안정";#N/A,#N/A,FALSE,"활동에 대한 안정";#N/A,#N/A,FALSE,"지지력 검토";#N/A,#N/A,FALSE,"PILE 계산";#N/A,#N/A,FALSE,"PILE계산결과";#N/A,#N/A,FALSE,"PILE검토";#N/A,#N/A,FALSE,"벽체의 설계"}</definedName>
     <definedName name="ㅂㅎ" hidden="1">{#N/A,#N/A,FALSE,"하중 계산 (1)";#N/A,#N/A,FALSE,"토압계수계산";#N/A,#N/A,FALSE,"횡토압계산";#N/A,#N/A,FALSE,"전도에 대한 안정";#N/A,#N/A,FALSE,"활동에 대한 안정";#N/A,#N/A,FALSE,"지지력 검토";#N/A,#N/A,FALSE,"PILE 계산";#N/A,#N/A,FALSE,"PILE계산결과";#N/A,#N/A,FALSE,"PILE검토";#N/A,#N/A,FALSE,"벽체의 설계"}</definedName>
     <definedName name="ㅂ호세">{"'표지'!$B$5"}</definedName>
-    <definedName name="바" localSheetId="0">BlankMacro1</definedName>
     <definedName name="바">BlankMacro1</definedName>
     <definedName name="바람">#REF!</definedName>
     <definedName name="바로" hidden="1">#REF!</definedName>
@@ -8551,12 +8495,10 @@
     <definedName name="바바바밥바바바바">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="바밥">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="바밥바">{"'5'!$A$1:$BB$147"}</definedName>
-    <definedName name="바보" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="바보">[0]!영광원자력5,#REF!</definedName>
     <definedName name="바보ㅗ옹아아러ㅏ">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="바부">{"'용역비'!$A$4:$C$8"}</definedName>
     <definedName name="바붕" hidden="1">{#N/A,#N/A,FALSE,"전력간선"}</definedName>
-    <definedName name="바탕화면" localSheetId="0">BlankMacro1</definedName>
     <definedName name="바탕화면">BlankMacro1</definedName>
     <definedName name="박" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="박보순" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
@@ -8580,12 +8522,10 @@
     <definedName name="밥바">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="밥바자">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="방류펌프">#REF!</definedName>
-    <definedName name="방배트윈품질" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="방배트윈품질">[0]!영광원자력5,#REF!</definedName>
     <definedName name="방부각재">931007</definedName>
     <definedName name="방부원주">1064010</definedName>
     <definedName name="방부판재">1037435</definedName>
-    <definedName name="방송" localSheetId="0">BlankMacro1</definedName>
     <definedName name="방송">BlankMacro1</definedName>
     <definedName name="방송설비">#REF!</definedName>
     <definedName name="방수" hidden="1">{#N/A,#N/A,TRUE,"토적및재료집계";#N/A,#N/A,TRUE,"토적및재료집계";#N/A,#N/A,TRUE,"단위량"}</definedName>
@@ -8593,7 +8533,6 @@
     <definedName name="방수시방1" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="방음벽" hidden="1">{#N/A,#N/A,FALSE,"배수2"}</definedName>
     <definedName name="방음벽번호">#REF!</definedName>
-    <definedName name="방이동" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="방이동">[0]!영광원자력5,#REF!</definedName>
     <definedName name="방진.도금">#REF!</definedName>
     <definedName name="배" hidden="1">{#N/A,#N/A,FALSE,"표지"}</definedName>
@@ -8770,7 +8709,6 @@
     <definedName name="부하">#REF!</definedName>
     <definedName name="분" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="분개표">{"서울냉천 3차( 5. 6-7).xls","Sheet1"}</definedName>
-    <definedName name="분뇨처리장장" localSheetId="0">BlankMacro1</definedName>
     <definedName name="분뇨처리장장">BlankMacro1</definedName>
     <definedName name="분당">#REF!</definedName>
     <definedName name="분당공" hidden="1">#REF!</definedName>
@@ -8806,11 +8744,8 @@
     <definedName name="분양" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="분양내역" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="분양별" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="분장실" localSheetId="0">BlankMacro1</definedName>
     <definedName name="분장실">BlankMacro1</definedName>
-    <definedName name="분전반" localSheetId="0">BlankMacro1</definedName>
     <definedName name="분전반">BlankMacro1</definedName>
-    <definedName name="분전반1" localSheetId="0">BlankMacro1</definedName>
     <definedName name="분전반1">BlankMacro1</definedName>
     <definedName name="분전반제조총괄표">{"'건축내역'!$A$1:$L$413"}</definedName>
     <definedName name="불광동" hidden="1">{#N/A,#N/A,FALSE,"포장2"}</definedName>
@@ -8959,14 +8894,12 @@
     <definedName name="산추">#REF!</definedName>
     <definedName name="산출">#REF!</definedName>
     <definedName name="산출1">#REF!</definedName>
-    <definedName name="산출근거" localSheetId="0">BlankMacro1</definedName>
     <definedName name="산출근거">BlankMacro1</definedName>
     <definedName name="산출근거1">#REF!</definedName>
     <definedName name="산출근거111">#REF!</definedName>
     <definedName name="산출금양">#REF!</definedName>
     <definedName name="산출내역">{"'단계별시설공사비'!$A$3:$K$51"}</definedName>
     <definedName name="산출서" hidden="1">{#N/A,#N/A,TRUE,"960318-1";#N/A,#N/A,TRUE,"960318-2";#N/A,#N/A,TRUE,"960318-3"}</definedName>
-    <definedName name="산출일위대가통신" localSheetId="0">BlankMacro1</definedName>
     <definedName name="산출일위대가통신">BlankMacro1</definedName>
     <definedName name="살수차">220000</definedName>
     <definedName name="삼">#REF!</definedName>
@@ -9099,14 +9032,11 @@
     <definedName name="소계5">#REF!</definedName>
     <definedName name="소공2">[0]!소공2</definedName>
     <definedName name="소모">#REF!</definedName>
-    <definedName name="소모품" localSheetId="0">Dlog_Show</definedName>
     <definedName name="소모품">Dlog_Show</definedName>
     <definedName name="소모품비">#REF!</definedName>
     <definedName name="소방" hidden="1">{"SJ - 기본 보기",#N/A,FALSE,"공사별 외주견적"}</definedName>
     <definedName name="소방감리">#REF!</definedName>
-    <definedName name="소방내역" localSheetId="0">BlankMacro1</definedName>
     <definedName name="소방내역">BlankMacro1</definedName>
-    <definedName name="소방내역서" localSheetId="0">BlankMacro1</definedName>
     <definedName name="소방내역서">BlankMacro1</definedName>
     <definedName name="소방사항" hidden="1">#REF!</definedName>
     <definedName name="소수력">{"'집계표'!$A$1:$F$40"}</definedName>
@@ -9173,13 +9103,10 @@
     <definedName name="수량검토">#REF!</definedName>
     <definedName name="수량계산">#REF!</definedName>
     <definedName name="수량산출">#REF!</definedName>
-    <definedName name="수량산출2" localSheetId="0">BlankMacro1</definedName>
     <definedName name="수량산출2">BlankMacro1</definedName>
-    <definedName name="수량산출5" localSheetId="0">BlankMacro1</definedName>
     <definedName name="수량산출5">BlankMacro1</definedName>
     <definedName name="수량산출서" hidden="1">#REF!</definedName>
     <definedName name="수량산출서2">#REF!</definedName>
-    <definedName name="수량산출서표지" localSheetId="0">BlankMacro1</definedName>
     <definedName name="수량산출서표지">BlankMacro1</definedName>
     <definedName name="수량입력">#REF!</definedName>
     <definedName name="수량조서1">#REF!</definedName>
@@ -9219,7 +9146,6 @@
     <definedName name="순공사비">#REF!</definedName>
     <definedName name="순공사비_현황">#REF!</definedName>
     <definedName name="순공사비계">#REF!</definedName>
-    <definedName name="순공사비산출서" localSheetId="0">Dlog_Show</definedName>
     <definedName name="순공사비산출서">Dlog_Show</definedName>
     <definedName name="순공사비집" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="순공사원가">#REF!</definedName>
@@ -9243,13 +9169,9 @@
     <definedName name="승인요청">#REF!</definedName>
     <definedName name="승호">#REF!</definedName>
     <definedName name="시">#REF!</definedName>
-    <definedName name="시3" localSheetId="0">BlankMacro1</definedName>
     <definedName name="시3">BlankMacro1</definedName>
-    <definedName name="시멘트" localSheetId="0">BlankMacro1</definedName>
     <definedName name="시멘트">BlankMacro1</definedName>
-    <definedName name="시멘트6" localSheetId="0">BlankMacro1</definedName>
     <definedName name="시멘트6">BlankMacro1</definedName>
-    <definedName name="시설" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="시설">[0]!영광원자력5,#REF!</definedName>
     <definedName name="시설물수량">#REF!</definedName>
     <definedName name="시설보강종합표">{"'집계표'!$A$1:$F$40"}</definedName>
@@ -9469,13 +9391,9 @@
     <definedName name="ㅇ화ㅓ랑러ㅣ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="ㅇ황히ㅗ이ㅓ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="아" hidden="1">#REF!</definedName>
-    <definedName name="아늘믿" localSheetId="0">BlankMacro1</definedName>
     <definedName name="아늘믿">BlankMacro1</definedName>
-    <definedName name="아니" localSheetId="0">BlankMacro1</definedName>
     <definedName name="아니">BlankMacro1</definedName>
-    <definedName name="아다" localSheetId="0">BlankMacro1</definedName>
     <definedName name="아다">BlankMacro1</definedName>
-    <definedName name="아디" localSheetId="0">BlankMacro1</definedName>
     <definedName name="아디">BlankMacro1</definedName>
     <definedName name="아라">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="아름" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
@@ -9484,7 +9402,6 @@
     <definedName name="아무" hidden="1">{#N/A,#N/A,FALSE,"배수2"}</definedName>
     <definedName name="아무거나" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="아무나" hidden="1">{#N/A,#N/A,FALSE,"토공2"}</definedName>
-    <definedName name="아서" localSheetId="0">BlankMacro1</definedName>
     <definedName name="아서">BlankMacro1</definedName>
     <definedName name="아스콘_기층_포설">#REF!</definedName>
     <definedName name="아스콘_포장깨기">#REF!</definedName>
@@ -9525,9 +9442,7 @@
     <definedName name="안성진행">#REF!</definedName>
     <definedName name="안성진행2">#REF!</definedName>
     <definedName name="안성청산">#REF!</definedName>
-    <definedName name="안양석수" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="안양석수">[0]!영광원자력5,#REF!</definedName>
-    <definedName name="안양석수1" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="안양석수1">[0]!영광원자력5,#REF!</definedName>
     <definedName name="안양현대" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="안전">#REF!</definedName>
@@ -9617,7 +9532,6 @@
     <definedName name="업체자료">#REF!</definedName>
     <definedName name="없음">{"'con_010'!$A$1:$AN$63"}</definedName>
     <definedName name="에" hidden="1">#REF!</definedName>
-    <definedName name="에로비" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="에로비">[0]!영광원자력5,#REF!</definedName>
     <definedName name="엑설">#REF!</definedName>
     <definedName name="여건22" hidden="1">#REF!</definedName>
@@ -9638,11 +9552,8 @@
     <definedName name="열교환기">#REF!</definedName>
     <definedName name="염색기술3" hidden="1">{#N/A,#N/A,TRUE,"손익보고"}</definedName>
     <definedName name="영" hidden="1">{#N/A,#N/A,FALSE,"표지"}</definedName>
-    <definedName name="영광" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="영광">[0]!영광원자력5,#REF!</definedName>
-    <definedName name="영광2" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="영광2">[0]!영광원자력5,#REF!</definedName>
-    <definedName name="영광원자력56호기" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="영광원자력56호기">[0]!영광원자력5,#REF!</definedName>
     <definedName name="영구배수견적특수조건" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="영남">#REF!</definedName>
@@ -9735,7 +9646,6 @@
     <definedName name="용동교" hidden="1">{#N/A,#N/A,FALSE,"배수1"}</definedName>
     <definedName name="용두동글로리" hidden="1">#REF!</definedName>
     <definedName name="용량">#REF!</definedName>
-    <definedName name="용마" localSheetId="0">BlankMacro1</definedName>
     <definedName name="용마">BlankMacro1</definedName>
     <definedName name="용소1_40">#REF!</definedName>
     <definedName name="용소2_25">#REF!</definedName>
@@ -9748,7 +9658,6 @@
     <definedName name="용접">#REF!</definedName>
     <definedName name="우" hidden="1">#REF!</definedName>
     <definedName name="우1탁1">{"'집계표'!$A$1:$F$40"}</definedName>
-    <definedName name="우띠" localSheetId="0">BlankMacro1</definedName>
     <definedName name="우띠">BlankMacro1</definedName>
     <definedName name="우리" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="우리나라" hidden="1">{#N/A,#N/A,FALSE,"전력간선"}</definedName>
@@ -9774,12 +9683,9 @@
     <definedName name="원">#REF!</definedName>
     <definedName name="원가" hidden="1">{#N/A,#N/A,FALSE,"운반시간"}</definedName>
     <definedName name="원가1" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
-    <definedName name="원가10" localSheetId="0">BlankMacro1</definedName>
     <definedName name="원가10">BlankMacro1</definedName>
-    <definedName name="원가12356987" localSheetId="0">BlankMacro1</definedName>
     <definedName name="원가12356987">BlankMacro1</definedName>
     <definedName name="원가계간" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="원가계산" localSheetId="0">Dlog_Show</definedName>
     <definedName name="원가계산">Dlog_Show</definedName>
     <definedName name="원가계산19" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="원가계산서">0</definedName>
@@ -9819,7 +9725,6 @@
     <definedName name="유리">#REF!</definedName>
     <definedName name="유리22MM" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="유병한">[0]!유병한</definedName>
-    <definedName name="유신" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="유신">[0]!영광원자력5,#REF!</definedName>
     <definedName name="유자">{"'표지'!$B$5"}</definedName>
     <definedName name="유정호" hidden="1">#REF!</definedName>
@@ -9874,7 +9779,6 @@
     <definedName name="이광훈9" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="이기성">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="이대GROSS">#N/A</definedName>
-    <definedName name="이런" localSheetId="0">BlankMacro1</definedName>
     <definedName name="이런">BlankMacro1</definedName>
     <definedName name="이름" hidden="1">{#N/A,#N/A,FALSE,"구조1"}</definedName>
     <definedName name="이름1" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
@@ -9924,7 +9828,6 @@
     <definedName name="인력" hidden="1">{#N/A,#N/A,TRUE,"표지";#N/A,#N/A,TRUE,"목차";#N/A,#N/A,TRUE,"1.0일반사항";#N/A,#N/A,TRUE,"2.0공급범위";#N/A,#N/A,TRUE,"3.0현장조건";#N/A,#N/A,TRUE,"4.0적용규격및표준";#N/A,#N/A,TRUE,"5.0요구조건";#N/A,#N/A,TRUE,"6.0시험및검사";#N/A,#N/A,TRUE,"7.0성능보장";#N/A,#N/A,TRUE,"8.0도장";#N/A,#N/A,TRUE,"9.0운송및납품";#N/A,#N/A,TRUE,"10예비품및공구";#N/A,#N/A,TRUE,"11대안";#N/A,#N/A,TRUE,"12제출자료";#N/A,#N/A,TRUE,"13입찰서양식";#N/A,#N/A,TRUE,"14첨부"}</definedName>
     <definedName name="인력기계" hidden="1">{#N/A,#N/A,TRUE,"표지";#N/A,#N/A,TRUE,"목차";#N/A,#N/A,TRUE,"1.0일반사항";#N/A,#N/A,TRUE,"2.0공급범위";#N/A,#N/A,TRUE,"3.0현장조건";#N/A,#N/A,TRUE,"4.0적용규격및표준";#N/A,#N/A,TRUE,"5.0요구조건";#N/A,#N/A,TRUE,"6.0시험및검사";#N/A,#N/A,TRUE,"7.0성능보장";#N/A,#N/A,TRUE,"8.0도장";#N/A,#N/A,TRUE,"9.0운송및납품";#N/A,#N/A,TRUE,"10예비품및공구";#N/A,#N/A,TRUE,"11대안";#N/A,#N/A,TRUE,"12제출자료";#N/A,#N/A,TRUE,"13입찰서양식";#N/A,#N/A,TRUE,"14첨부"}</definedName>
     <definedName name="인력품">#REF!</definedName>
-    <definedName name="인상익" localSheetId="0">BlankMacro1</definedName>
     <definedName name="인상익">BlankMacro1</definedName>
     <definedName name="인서트">#REF!</definedName>
     <definedName name="인쇄1">#REF!</definedName>
@@ -9936,7 +9839,6 @@
     <definedName name="인숭">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="인양제내역서">#REF!</definedName>
     <definedName name="인원">#REF!</definedName>
-    <definedName name="인원장비" localSheetId="0">BlankMacro1</definedName>
     <definedName name="인원장비">BlankMacro1</definedName>
     <definedName name="인원조직" hidden="1">0</definedName>
     <definedName name="인입비">#N/A</definedName>
@@ -10088,7 +9990,6 @@
     <definedName name="ㅈㅇㅀ" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="ㅈㅈ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="ㅈㅈㄷㅈ">{"'표지'!$B$5"}</definedName>
-    <definedName name="ㅈㅈㅂㅈ" localSheetId="0">BlankMacro1</definedName>
     <definedName name="ㅈㅈㅂㅈ">BlankMacro1</definedName>
     <definedName name="ㅈㅈㅈ">{"'용역비'!$A$4:$C$8"}</definedName>
     <definedName name="ㅈㅈㅈㅈ" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
@@ -10097,7 +9998,6 @@
     <definedName name="자" hidden="1">{#N/A,#N/A,FALSE,"UNIT";#N/A,#N/A,FALSE,"UNIT";#N/A,#N/A,FALSE,"계정"}</definedName>
     <definedName name="자." hidden="1">{#N/A,#N/A,FALSE,"UNIT";#N/A,#N/A,FALSE,"UNIT";#N/A,#N/A,FALSE,"계정"}</definedName>
     <definedName name="자.." hidden="1">{#N/A,#N/A,FALSE,"UNIT";#N/A,#N/A,FALSE,"UNIT";#N/A,#N/A,FALSE,"계정"}</definedName>
-    <definedName name="자3" localSheetId="0">BlankMacro1</definedName>
     <definedName name="자3">BlankMacro1</definedName>
     <definedName name="자38">#REF!</definedName>
     <definedName name="자60">#REF!</definedName>
@@ -10112,10 +10012,8 @@
     <definedName name="자다라다">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="자다라다가라">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="자다라다라다라">{"'5'!$A$1:$BB$147"}</definedName>
-    <definedName name="자동제어" localSheetId="0">BlankMacro1</definedName>
     <definedName name="자동제어">BlankMacro1</definedName>
     <definedName name="자동제어.도급">#REF!</definedName>
-    <definedName name="자동제어1차공량산출" localSheetId="0">BlankMacro1</definedName>
     <definedName name="자동제어1차공량산출">BlankMacro1</definedName>
     <definedName name="자동화재탐지설비">#REF!</definedName>
     <definedName name="자료1">#REF!</definedName>
@@ -10254,13 +10152,10 @@
     <definedName name="전기구" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="전기기기">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="전기내역" hidden="1">{#N/A,#N/A,FALSE,"CCTV"}</definedName>
-    <definedName name="전기내역3" localSheetId="0">BlankMacro1</definedName>
     <definedName name="전기내역3">BlankMacro1</definedName>
     <definedName name="전기내역서">#REF!</definedName>
     <definedName name="전기마감" hidden="1">#REF!</definedName>
-    <definedName name="전기변경1" localSheetId="0">BlankMacro1</definedName>
     <definedName name="전기변경1">BlankMacro1</definedName>
-    <definedName name="전기변경3" localSheetId="0">BlankMacro1</definedName>
     <definedName name="전기변경3">BlankMacro1</definedName>
     <definedName name="전기서비스">#N/A</definedName>
     <definedName name="전기집계">#REF!</definedName>
@@ -10293,7 +10188,6 @@
     <definedName name="전체">#REF!</definedName>
     <definedName name="전체공정표" hidden="1">{#N/A,#N/A,TRUE,"단가산출서";#N/A,#N/A,TRUE,"수량산출서"}</definedName>
     <definedName name="전체공종">#REF!</definedName>
-    <definedName name="전체대비예상" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="전체대비예상">[0]!영광원자력5,#REF!</definedName>
     <definedName name="전체제조총괄표">{"'건축내역'!$A$1:$L$413"}</definedName>
     <definedName name="전체평단가">#REF!</definedName>
@@ -10406,9 +10300,7 @@
     <definedName name="조정금액" hidden="1">#REF!</definedName>
     <definedName name="조정요율" hidden="1">#REF!</definedName>
     <definedName name="조조" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
-    <definedName name="조조조조" localSheetId="0">BlankMacro1</definedName>
     <definedName name="조조조조">BlankMacro1</definedName>
-    <definedName name="조조조조좆" localSheetId="0">BlankMacro1</definedName>
     <definedName name="조조조조좆">BlankMacro1</definedName>
     <definedName name="조직도" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="조직인원" hidden="1">0</definedName>
@@ -10428,7 +10320,6 @@
     <definedName name="종배수관부설">#REF!</definedName>
     <definedName name="종자" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="종합청사" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="종현" localSheetId="0">BlankMacro1</definedName>
     <definedName name="종현">BlankMacro1</definedName>
     <definedName name="죠" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="죠ㅓㅈ겨ㅗ굦" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
@@ -10487,7 +10378,6 @@
     <definedName name="지입수불대장이동">#REF!</definedName>
     <definedName name="지입재료비">#REF!</definedName>
     <definedName name="지적사항">#REF!</definedName>
-    <definedName name="지주목" localSheetId="0">BlankMacro1</definedName>
     <definedName name="지주목">BlankMacro1</definedName>
     <definedName name="지중" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="지철" hidden="1">{#N/A,#N/A,FALSE,"포장2"}</definedName>
@@ -10505,7 +10395,6 @@
     <definedName name="직노_1">#REF!</definedName>
     <definedName name="직노_2">#REF!</definedName>
     <definedName name="직매54P" hidden="1">{#N/A,#N/A,TRUE,"토적및재료집계";#N/A,#N/A,TRUE,"토적및재료집계";#N/A,#N/A,TRUE,"단위량"}</definedName>
-    <definedName name="직원발령요청" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="직원발령요청">[0]!영광원자력5,#REF!</definedName>
     <definedName name="직원소요철수계획" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="직원조직" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
@@ -10563,7 +10452,6 @@
     <definedName name="ㅊㅍㅋㅌㅍㅌ" hidden="1">{#N/A,#N/A,FALSE,"혼합골재"}</definedName>
     <definedName name="ㅊㅍㅌ" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="ㅊㅍㅍ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="차" localSheetId="0">BlankMacro1</definedName>
     <definedName name="차">BlankMacro1</definedName>
     <definedName name="차." hidden="1">{#N/A,#N/A,FALSE,"UNIT";#N/A,#N/A,FALSE,"UNIT";#N/A,#N/A,FALSE,"계정"}</definedName>
     <definedName name="차도1호갯수">#REF!</definedName>
@@ -10585,11 +10473,9 @@
     <definedName name="천사">{"'용역비'!$A$4:$C$8"}</definedName>
     <definedName name="철2" hidden="1">{#N/A,#N/A,FALSE,"혼합골재"}</definedName>
     <definedName name="철간">#REF!</definedName>
-    <definedName name="철거" localSheetId="0">BlankMacro1</definedName>
     <definedName name="철거">BlankMacro1</definedName>
     <definedName name="철거2" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="철거공사비">#N/A</definedName>
-    <definedName name="철거공사산출서" localSheetId="0">BlankMacro1</definedName>
     <definedName name="철거공사산출서">BlankMacro1</definedName>
     <definedName name="철거산출근거서">#REF!</definedName>
     <definedName name="철거자재">#REF!</definedName>
@@ -10608,7 +10494,6 @@
     <definedName name="철근공사예산안" hidden="1">{#N/A,#N/A,TRUE,"토적및재료집계";#N/A,#N/A,TRUE,"토적및재료집계";#N/A,#N/A,TRUE,"단위량"}</definedName>
     <definedName name="철근수정본">{"'Sheet1'!$A$4:$M$21","'Sheet1'!$J$17:$K$19"}</definedName>
     <definedName name="철립">#REF!</definedName>
-    <definedName name="철물갑지" localSheetId="0">Dlog_Show</definedName>
     <definedName name="철물갑지">Dlog_Show</definedName>
     <definedName name="철재류_운반">#REF!</definedName>
     <definedName name="철재류운반">#REF!</definedName>
@@ -10636,13 +10521,11 @@
     <definedName name="총괄1" hidden="1">{#N/A,#N/A,TRUE,"총괄"}</definedName>
     <definedName name="총괄2" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="총괄7" hidden="1">{#N/A,#N/A,FALSE,"앞";#N/A,#N/A,FALSE,"앞";#N/A,#N/A,FALSE,"목차";#N/A,#N/A,FALSE,"1";#N/A,#N/A,FALSE,"갑지";#N/A,#N/A,FALSE,"2";#N/A,#N/A,FALSE,"개요";#N/A,#N/A,FALSE,"개요2";#N/A,#N/A,FALSE,"3";#N/A,#N/A,FALSE,"총괄";#N/A,#N/A,FALSE,"선금";#N/A,#N/A,FALSE,"4";#N/A,#N/A,FALSE,"방법";#N/A,#N/A,FALSE,"5";#N/A,#N/A,FALSE,"k";#N/A,#N/A,FALSE,"6";#N/A,#N/A,FALSE,"지수";#N/A,#N/A,FALSE,"7";#N/A,#N/A,FALSE,"노";#N/A,#N/A,FALSE,"경";#N/A,#N/A,FALSE,"재";#N/A,#N/A,FALSE,"산";#N/A,#N/A,FALSE,"안";#N/A,#N/A,FALSE,"8";#N/A,#N/A,FALSE,"계수";#N/A,#N/A,FALSE,"9";#N/A,#N/A,FALSE,"비목";#N/A,#N/A,FALSE,"10";#N/A,#N/A,FALSE,"집계"}</definedName>
-    <definedName name="총괄갑지" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="총괄갑지">[0]!영광원자력5,#REF!</definedName>
     <definedName name="총괄공사예산서">#REF!</definedName>
     <definedName name="총괄제출용" hidden="1">{#N/A,#N/A,FALSE,"전력간선"}</definedName>
     <definedName name="총괄집계" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="총괄표" hidden="1">#REF!</definedName>
-    <definedName name="총괄표2" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="총괄표2">[0]!영광원자력5,#REF!</definedName>
     <definedName name="총괄표3" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
     <definedName name="총괄표9층">#REF!</definedName>
@@ -10804,36 +10687,21 @@
     <definedName name="테이블1">#REF!</definedName>
     <definedName name="테이블2">#REF!</definedName>
     <definedName name="텍코팅">#REF!</definedName>
-    <definedName name="템" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템">BlankMacro1</definedName>
-    <definedName name="템2" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템2">BlankMacro1</definedName>
-    <definedName name="템3" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템3">BlankMacro1</definedName>
-    <definedName name="템4" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템4">BlankMacro1</definedName>
-    <definedName name="템5" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템5">BlankMacro1</definedName>
-    <definedName name="템6" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템6">BlankMacro1</definedName>
-    <definedName name="템플리트모듈1" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템플리트모듈1">BlankMacro1</definedName>
-    <definedName name="템플리트모듈10" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템플리트모듈10">BlankMacro1</definedName>
-    <definedName name="템플리트모듈2" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템플리트모듈2">BlankMacro1</definedName>
-    <definedName name="템플리트모듈3" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템플리트모듈3">BlankMacro1</definedName>
-    <definedName name="템플리트모듈33" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템플리트모듈33">BlankMacro1</definedName>
-    <definedName name="템플리트모듈4" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템플리트모듈4">BlankMacro1</definedName>
-    <definedName name="템플리트모듈5" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템플리트모듈5">BlankMacro1</definedName>
-    <definedName name="템플리트모듈6" localSheetId="0">BlankMacro1</definedName>
     <definedName name="템플리트모듈6">BlankMacro1</definedName>
     <definedName name="토" hidden="1">#REF!</definedName>
-    <definedName name="토3" localSheetId="0">BlankMacro1</definedName>
     <definedName name="토3">BlankMacro1</definedName>
     <definedName name="토건" hidden="1">{"'장비'!$A$3:$M$12"}</definedName>
     <definedName name="토건공사비대비r">{"'장비'!$A$3:$M$12"}</definedName>
@@ -11003,7 +10871,6 @@
     <definedName name="파일견적용">[0]!파일견적용</definedName>
     <definedName name="파일본수">#REF!</definedName>
     <definedName name="파일산출3" hidden="1">#REF!</definedName>
-    <definedName name="파일수량2" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="파일수량2">[0]!영광원자력5,#REF!</definedName>
     <definedName name="파자다라달">{"'5'!$A$1:$BB$147"}</definedName>
     <definedName name="파주보고최종4.26" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
@@ -11029,11 +10896,9 @@
     <definedName name="폐기물_운반">#REF!</definedName>
     <definedName name="폐기물_저장창고_및_소각로">#REF!</definedName>
     <definedName name="폐기물_처리비">#REF!</definedName>
-    <definedName name="폐기물내역서" localSheetId="0">template!템플리트모듈6</definedName>
     <definedName name="폐기물내역서">[0]!템플리트모듈6</definedName>
     <definedName name="폐기물산출내역서" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="폐기물수수료">#REF!</definedName>
-    <definedName name="폐기물예산" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="폐기물예산">[0]!영광원자력5,#REF!</definedName>
     <definedName name="폐기물운반">#REF!</definedName>
     <definedName name="폐기물집계표">[0]!집</definedName>
@@ -11043,9 +10908,7 @@
     <definedName name="포설노무비">#REF!</definedName>
     <definedName name="포장2월ocf" hidden="1">{#N/A,#N/A,FALSE,"지침";#N/A,#N/A,FALSE,"환경분석";#N/A,#N/A,FALSE,"Sheet16"}</definedName>
     <definedName name="포장ocf" hidden="1">{#N/A,#N/A,FALSE,"지침";#N/A,#N/A,FALSE,"환경분석";#N/A,#N/A,FALSE,"Sheet16"}</definedName>
-    <definedName name="포장공" localSheetId="0">BlankMacro1</definedName>
     <definedName name="포장공">BlankMacro1</definedName>
-    <definedName name="포장공1" localSheetId="0">BlankMacro1</definedName>
     <definedName name="포장공1">BlankMacro1</definedName>
     <definedName name="포천주공임시">#REF!</definedName>
     <definedName name="포항내역서">#REF!</definedName>
@@ -11061,7 +10924,6 @@
     <definedName name="표준일위">#REF!</definedName>
     <definedName name="표지" hidden="1">#REF!</definedName>
     <definedName name="표지1" hidden="1">#REF!</definedName>
-    <definedName name="표지14" localSheetId="0">BlankMacro1</definedName>
     <definedName name="표지14">BlankMacro1</definedName>
     <definedName name="표지2" hidden="1">#REF!</definedName>
     <definedName name="표지3" hidden="1">{#N/A,#N/A,FALSE,"이정표"}</definedName>
@@ -11082,7 +10944,6 @@
     <definedName name="품셈단가">#REF!</definedName>
     <definedName name="품셈단가표">#REF!</definedName>
     <definedName name="품셈표준">#REF!</definedName>
-    <definedName name="품위내역서" localSheetId="0">BlankMacro1</definedName>
     <definedName name="품위내역서">BlankMacro1</definedName>
     <definedName name="품의민원" hidden="1">{#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"조직표";#N/A,#N/A,FALSE,"정직원인원";#N/A,#N/A,FALSE,"사업계획";#N/A,#N/A,FALSE,"부동산";#N/A,#N/A,FALSE,"장비현황";#N/A,#N/A,FALSE,"장비가동";#N/A,#N/A,FALSE,"매각장비";#N/A,#N/A,FALSE,"철구제작";#N/A,#N/A,FALSE,"철구수주";#N/A,#N/A,FALSE,"철구시설";#N/A,#N/A,FALSE,"준설장비";#N/A,#N/A,FALSE,"준설수량";#N/A,#N/A,FALSE,"골재인원";#N/A,#N/A,FALSE,"골재손익";#N/A,#N/A,FALSE,"노조현황"}</definedName>
     <definedName name="품의서1" hidden="1">#REF!</definedName>
@@ -11130,7 +10991,6 @@
     <definedName name="ㅎㄹㄴㄺ" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="ㅎㄹㄴㅇ" hidden="1">{#N/A,#N/A,FALSE,"단가표지"}</definedName>
     <definedName name="ㅎㄹㄷ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
-    <definedName name="ㅎㄹㅇ" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ㅎㄹㅇ">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ㅎㄹㅇㄴ" hidden="1">{#N/A,#N/A,FALSE,"골재소요량";#N/A,#N/A,FALSE,"골재소요량"}</definedName>
     <definedName name="ㅎㄹㅇㅁㅁㅎ" hidden="1">{#N/A,#N/A,FALSE,"조골재"}</definedName>
@@ -11178,7 +11038,6 @@
     <definedName name="ㅎㅇㅀㅇㅀㅇ" hidden="1">{#N/A,#N/A,FALSE,"표지목차"}</definedName>
     <definedName name="ㅎㅇㅁㄴㄹ" hidden="1">{#N/A,#N/A,FALSE,"운반시간"}</definedName>
     <definedName name="ㅎㅇㅁㅀㅁㅇ" hidden="1">{#N/A,#N/A,FALSE,"단가표지"}</definedName>
-    <definedName name="ㅎㅇㅎㅇㅎ" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ㅎㅇㅎㅇㅎ">[0]!영광원자력5,#REF!</definedName>
     <definedName name="ㅎ아라ㅣㅛㅕ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
     <definedName name="ㅎ오">{"'용역비'!$A$4:$C$8"}</definedName>
@@ -11228,7 +11087,6 @@
     <definedName name="한전수" hidden="1">{#N/A,#N/A,FALSE,"명세표"}</definedName>
     <definedName name="한전수탁비">#REF!</definedName>
     <definedName name="한타" hidden="1">{#N/A,#N/A,FALSE,"현장 NCR 분석";#N/A,#N/A,FALSE,"현장품질감사";#N/A,#N/A,FALSE,"현장품질감사"}</definedName>
-    <definedName name="한타공기" localSheetId="0">[0]!영광원자력5,#REF!</definedName>
     <definedName name="한타공기">[0]!영광원자력5,#REF!</definedName>
     <definedName name="할마버지" hidden="1">{#N/A,#N/A,FALSE,"이태원철근"}</definedName>
     <definedName name="할ㅇㅎㅎ랄ㄴㅇ험ㄴ히ㅓ" hidden="1">{#N/A,#N/A,FALSE,"총괄표지";#N/A,#N/A,FALSE,"표지";#N/A,#N/A,FALSE,"총표지";#N/A,#N/A,FALSE,"집계(총괄)";#N/A,#N/A,FALSE,"집계(토목)";#N/A,#N/A,FALSE,"집계 (R.C)";#N/A,#N/A,FALSE,"집계(철골)";#N/A,#N/A,FALSE,"집계(PC)";#N/A,#N/A,FALSE,"지급자재";#N/A,#N/A,FALSE,"RC";#N/A,#N/A,FALSE,"철골";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"PC";#N/A,#N/A,FALSE,"하도급총괄표";#N/A,#N/A,FALSE,"하도급사항";#N/A,#N/A,FALSE,"하도급산출내역별지";#N/A,#N/A,FALSE,"세부표지";#N/A,#N/A,FALSE,"부대입찰에 관한 확약서";#N/A,#N/A,FALSE,"토목"}</definedName>
@@ -11817,15 +11675,15 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>사용기간 : 2026년 5월 1일 ~ 2026년 5월 31일</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>정산인 : 김 복 수 (인)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>사용자 : 김 복 수</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>사용기간 : 2026년 6월 1일 ~ 2026년 6월 30일</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -11940,7 +11798,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -12217,43 +12075,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="dotted">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="dotted">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -12264,7 +12085,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFill="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -12374,24 +12195,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -12728,7 +12531,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87B85934-C0FE-4E2F-973C-294C31AC1B8D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{928A92ED-425E-4C67-98F6-A96616192EC0}">
   <sheetPr>
     <tabColor theme="4" tint="0.79998168889431442"/>
     <pageSetUpPr fitToPage="1"/>
@@ -13264,12 +13067,12 @@
     </row>
     <row r="2" spans="1:7" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="10"/>
       <c r="G2" s="11" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -13323,8 +13126,8 @@
         <f>ROW()-3</f>
         <v>3</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="41"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="34"/>
       <c r="D6" s="34"/>
       <c r="E6" s="35"/>
       <c r="F6" s="37"/>
@@ -13335,8 +13138,8 @@
         <f>ROW()-3</f>
         <v>4</v>
       </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="42"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="34"/>
       <c r="D7" s="34"/>
       <c r="E7" s="35"/>
       <c r="F7" s="37"/>
@@ -13347,8 +13150,8 @@
         <f>ROW()-3</f>
         <v>5</v>
       </c>
-      <c r="B8" s="39"/>
-      <c r="C8" s="42"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="34"/>
       <c r="D8" s="34"/>
       <c r="E8" s="35"/>
       <c r="F8" s="37"/>
@@ -13359,8 +13162,8 @@
         <f>ROW()-3</f>
         <v>6</v>
       </c>
-      <c r="B9" s="39"/>
-      <c r="C9" s="42"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="34"/>
       <c r="D9" s="34"/>
       <c r="E9" s="35"/>
       <c r="F9" s="37"/>
@@ -13371,8 +13174,8 @@
         <f>ROW()-3</f>
         <v>7</v>
       </c>
-      <c r="B10" s="40"/>
-      <c r="C10" s="43"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="34"/>
       <c r="D10" s="34"/>
       <c r="E10" s="35"/>
       <c r="F10" s="37"/>
@@ -13802,7 +13605,7 @@
     </row>
     <row r="46" spans="1:7" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="G46" s="11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -13818,10 +13621,6 @@
     <row r="57" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <mergeCells count="2">
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="C6:C10"/>
-  </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.35433070866141736" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>